<commit_message>
Version that can run battery data
</commit_message>
<xml_diff>
--- a/docs/Files/ODYM_Classifications_LL.xlsx
+++ b/docs/Files/ODYM_Classifications_LL.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA352843-380A-4B73-AAAD-BFACE8509DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E522AE9-AE47-417F-8A56-070DF0006C51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover_Dimensions_Aspects" sheetId="8" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="283">
   <si>
     <t>Name</t>
   </si>
@@ -791,9 +791,6 @@
     <t>India</t>
   </si>
   <si>
-    <t>Stefan Pauliuk, 2019</t>
-  </si>
-  <si>
     <t>3b0b3a88-864c-4acf-a00a-29eb80e060be</t>
   </si>
   <si>
@@ -851,12 +848,6 @@
     <t>d70ff49d-88c3-4a52-a12e-14ec6f53984f</t>
   </si>
   <si>
-    <t>construction</t>
-  </si>
-  <si>
-    <t>products and other</t>
-  </si>
-  <si>
     <t>Scenario</t>
   </si>
   <si>
@@ -894,6 +885,9 @@
   </si>
   <si>
     <t>Other scrap</t>
+  </si>
+  <si>
+    <t>Liz Lanphear, 2025</t>
   </si>
 </sst>
 </file>
@@ -1361,7 +1355,7 @@
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
-        <v>250</v>
+        <v>282</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.35">
@@ -1369,7 +1363,7 @@
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
@@ -1377,7 +1371,7 @@
         <v>3</v>
       </c>
       <c r="C7" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.35">
@@ -1944,10 +1938,6 @@
         <f>Chemical_Elements!D4</f>
         <v>He</v>
       </c>
-      <c r="F13" t="str">
-        <f>End_Use_Sectors!D4</f>
-        <v>construction</v>
-      </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="6">
@@ -1960,10 +1950,6 @@
       <c r="D14" t="str">
         <f>Chemical_Elements!D5</f>
         <v>Li</v>
-      </c>
-      <c r="F14" t="str">
-        <f>End_Use_Sectors!D5</f>
-        <v>products and other</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.35">
@@ -25709,7 +25695,7 @@
     </row>
     <row r="103" spans="4:6" x14ac:dyDescent="0.35">
       <c r="D103" s="4" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E103">
         <v>101</v>
@@ -25736,7 +25722,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>10</v>
@@ -25757,7 +25743,7 @@
         <v>13</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -25769,10 +25755,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -25787,7 +25773,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E4">
         <v>2</v>
@@ -25799,10 +25785,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E5">
         <v>3</v>
@@ -25817,7 +25803,7 @@
         <v>43487</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E6">
         <v>4</v>
@@ -25832,7 +25818,7 @@
         <v>43487</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E7">
         <v>5</v>
@@ -25869,7 +25855,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D10" s="4" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E10">
         <v>8</v>
@@ -25878,7 +25864,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D11" s="4" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E11">
         <v>9</v>
@@ -25887,7 +25873,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D12" s="4" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E12">
         <v>10</v>
@@ -26272,7 +26258,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>10</v>
@@ -26292,7 +26278,7 @@
         <v>224</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -26307,7 +26293,7 @@
         <v>246</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -26329,7 +26315,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D5" s="1"/>
       <c r="F5" s="1"/>
@@ -26458,7 +26444,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>10</v>
@@ -26479,7 +26465,7 @@
         <v>224</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -26494,7 +26480,7 @@
         <v>239</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -26508,12 +26494,7 @@
       <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
+      <c r="D4" s="1"/>
       <c r="F4" s="1"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -26521,14 +26502,9 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>268</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="E5">
-        <v>3</v>
-      </c>
+        <v>267</v>
+      </c>
+      <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
@@ -26655,7 +26631,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>10</v>
@@ -26675,7 +26651,7 @@
         <v>224</v>
       </c>
       <c r="D2" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -26692,7 +26668,7 @@
         <v>240</v>
       </c>
       <c r="D3" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -26716,7 +26692,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F5" s="1"/>
       <c r="H5" s="1"/>
@@ -26858,7 +26834,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>10</v>
@@ -26875,10 +26851,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
+        <v>269</v>
+      </c>
+      <c r="D2" t="s">
         <v>272</v>
-      </c>
-      <c r="D2" t="s">
-        <v>275</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -26891,10 +26867,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="D3" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -26917,7 +26893,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="F5" s="1"/>
       <c r="H5" s="1"/>

</xml_diff>